<commit_message>
chore(data-release): publish site data 2026-08-22 02:00:26 UTC
</commit_message>
<xml_diff>
--- a/diseases/d004/2026-2029.xlsx
+++ b/diseases/d004/2026-2029.xlsx
@@ -24670,13 +24670,13 @@
         </is>
       </c>
       <c r="N142" t="n">
-        <v>6113</v>
+        <v>6493</v>
       </c>
       <c r="O142" t="n">
-        <v>6113</v>
+        <v>6493</v>
       </c>
       <c r="R142" t="n">
-        <v>22.45189865272448</v>
+        <v>23.847567144142</v>
       </c>
       <c r="S142" t="inlineStr">
         <is>
@@ -24815,13 +24815,13 @@
         </is>
       </c>
       <c r="N143" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="O143" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="R143" t="n">
-        <v>0.1245166419604896</v>
+        <v>0.1600928253777724</v>
       </c>
       <c r="S143" t="inlineStr">
         <is>
@@ -24974,10 +24974,10 @@
         </is>
       </c>
       <c r="N144" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="O144" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="U144" t="inlineStr">
         <is>
@@ -25609,7 +25609,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>935318</v>
+        <v>935700</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-08-24 01:52:39 UTC
</commit_message>
<xml_diff>
--- a/diseases/d004/2026-2029.xlsx
+++ b/diseases/d004/2026-2029.xlsx
@@ -24670,13 +24670,13 @@
         </is>
       </c>
       <c r="N142" t="n">
-        <v>6661</v>
+        <v>6778</v>
       </c>
       <c r="O142" t="n">
-        <v>6661</v>
+        <v>6778</v>
       </c>
       <c r="R142" t="n">
-        <v>24.46459952982132</v>
+        <v>24.89431851270514</v>
       </c>
       <c r="S142" t="inlineStr">
         <is>
@@ -25609,7 +25609,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>935868</v>
+        <v>935985</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-08-25 02:00:27 UTC
</commit_message>
<xml_diff>
--- a/diseases/d004/2026-2029.xlsx
+++ b/diseases/d004/2026-2029.xlsx
@@ -24670,13 +24670,13 @@
         </is>
       </c>
       <c r="N142" t="n">
-        <v>6778</v>
+        <v>7176</v>
       </c>
       <c r="O142" t="n">
-        <v>6778</v>
+        <v>7176</v>
       </c>
       <c r="R142" t="n">
-        <v>24.89431851270514</v>
+        <v>26.35609761687402</v>
       </c>
       <c r="S142" t="inlineStr">
         <is>
@@ -25609,7 +25609,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>935985</v>
+        <v>936383</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-09-05 06:47:13 UTC
</commit_message>
<xml_diff>
--- a/diseases/d004/2026-2029.xlsx
+++ b/diseases/d004/2026-2029.xlsx
@@ -27480,13 +27480,13 @@
         </is>
       </c>
       <c r="N161" t="n">
-        <v>9697</v>
+        <v>9714</v>
       </c>
       <c r="O161" t="n">
-        <v>9697</v>
+        <v>9714</v>
       </c>
       <c r="R161" t="n">
-        <v>35.61525621388341</v>
+        <v>35.67769401481524</v>
       </c>
       <c r="S161" t="inlineStr">
         <is>
@@ -29734,13 +29734,13 @@
         </is>
       </c>
       <c r="N176" t="n">
-        <v>319</v>
+        <v>639</v>
       </c>
       <c r="O176" t="n">
-        <v>319</v>
+        <v>639</v>
       </c>
       <c r="R176" t="n">
-        <v>1.171626970426813</v>
+        <v>2.346926752673146</v>
       </c>
       <c r="S176" t="inlineStr">
         <is>
@@ -30383,7 +30383,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>975149</v>
+        <v>975486</v>
       </c>
     </row>
     <row r="16">

</xml_diff>